<commit_message>
Add dashboard file timestamps, user permissions system, and Orders Backlog Admin tab
- SAP Reports dashboard now shows file modification date/time for all input and output files
- PDF generation already includes date+time from input file directory timestamp
- Orders Backlog: new Admin tab with Users, Contract Types, Companies management
- User permissions system: 6 module-level Edit/Read permissions stored in users.xlsx
- Admin tab restricted to Admin-role users only
- Session API endpoint for frontend permission checks
- Collapsible month sections on SAP Reports dashboard
- Aggregate P&L Output restored to dashboard with download button
- Fixed file auto-sorting on upload
- PROJECT_CONTEXT.md added for project documentation

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/SAP Reports/Annual Financial Data/Aggregate P&L Output.xlsx
+++ b/SAP Reports/Annual Financial Data/Aggregate P&L Output.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1" refMode="A1" iterate="0" iterateCount="100" iterateDelta="0.0001"/>
@@ -808,13 +808,13 @@
         </is>
       </c>
       <c r="C7" s="20" t="n">
-        <v>0</v>
+        <v>1858364.25</v>
       </c>
       <c r="D7" s="20" t="n">
-        <v>0</v>
+        <v>1640834.72</v>
       </c>
       <c r="E7" s="20" t="n">
-        <v>200456.92</v>
+        <v>898497.73</v>
       </c>
       <c r="F7" s="20" t="n">
         <v>0</v>
@@ -859,13 +859,13 @@
         </is>
       </c>
       <c r="C8" s="20" t="n">
-        <v>0</v>
+        <v>-1265003.14</v>
       </c>
       <c r="D8" s="20" t="n">
-        <v>0</v>
+        <v>-1072556.73</v>
       </c>
       <c r="E8" s="20" t="n">
-        <v>-8185.92</v>
+        <v>-51022.43</v>
       </c>
       <c r="F8" s="20" t="n">
         <v>0</v>
@@ -910,13 +910,13 @@
         </is>
       </c>
       <c r="C9" s="20" t="n">
-        <v>-117764.65</v>
+        <v>-224269.83</v>
       </c>
       <c r="D9" s="20" t="n">
-        <v>-175096.25</v>
+        <v>-264679.16</v>
       </c>
       <c r="E9" s="20" t="n">
-        <v>0</v>
+        <v>-106813.86</v>
       </c>
       <c r="F9" s="20" t="n">
         <v>-1800</v>
@@ -961,13 +961,13 @@
         </is>
       </c>
       <c r="C10" s="20" t="n">
-        <v>-158601.03</v>
+        <v>329164.9</v>
       </c>
       <c r="D10" s="20" t="n">
-        <v>-178282.4</v>
+        <v>289650.96</v>
       </c>
       <c r="E10" s="20" t="n">
-        <v>192271</v>
+        <v>330661.44</v>
       </c>
       <c r="F10" s="20" t="n">
         <v>-1800</v>
@@ -979,7 +979,7 @@
         <v>-4816.5</v>
       </c>
       <c r="I10" s="20" t="n">
-        <v>-261125.88</v>
+        <v>-372961.04</v>
       </c>
       <c r="J10" s="20" t="n">
         <v>-9615.209999999999</v>
@@ -1012,13 +1012,13 @@
         </is>
       </c>
       <c r="C11" s="24" t="n">
-        <v>-158601.03</v>
+        <v>329164.9</v>
       </c>
       <c r="D11" s="24" t="n">
-        <v>-179702.4</v>
+        <v>286810.96</v>
       </c>
       <c r="E11" s="24" t="n">
-        <v>192271</v>
+        <v>330661.44</v>
       </c>
       <c r="F11" s="24" t="n">
         <v>-1800</v>
@@ -1030,7 +1030,7 @@
         <v>-4816.5</v>
       </c>
       <c r="I11" s="24" t="n">
-        <v>-261125.88</v>
+        <v>-372961.04</v>
       </c>
       <c r="J11" s="24" t="n">
         <v>-9615.209999999999</v>

</xml_diff>